<commit_message>
Increment version to 18.0.1.0.14. Update summary report template and enhance Excel report generation by adding functionality to clear summary data rows and calculate totals dynamically. Adjusted the layout to maintain merged header/footer integrity during report generation.
</commit_message>
<xml_diff>
--- a/rgb_workover_operations/report/excel_templates/summary_report_template.xlsx
+++ b/rgb_workover_operations/report/excel_templates/summary_report_template.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy;@"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -495,7 +494,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -576,7 +575,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -638,6 +637,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1015,8 +1017,13 @@
     <col width="8.33203125" customWidth="1" min="7" max="7"/>
     <col width="9.6640625" customWidth="1" min="8" max="8"/>
     <col width="15.44140625" customWidth="1" min="9" max="9"/>
-    <col width="162.5546875" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
     <col width="3.44140625" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
   </cols>
@@ -1062,12 +1069,12 @@
       <c r="G2" s="10" t="n"/>
       <c r="H2" s="10" t="n"/>
       <c r="I2" s="10" t="n"/>
-      <c r="J2" s="11" t="inlineStr">
+      <c r="J2" s="11" t="n"/>
+      <c r="K2" t="inlineStr">
         <is>
-          <t>Month of  ( MAY-2026 )</t>
+          <t>Month of  (  )</t>
         </is>
       </c>
-      <c r="Q2" s="12" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="13" t="n"/>
@@ -1079,7 +1086,6 @@
       <c r="G3" s="14" t="n"/>
       <c r="H3" s="14" t="n"/>
       <c r="I3" s="14" t="n"/>
-      <c r="Q3" s="12" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="15" t="n"/>
@@ -1115,18 +1121,12 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="J4" s="21" t="inlineStr">
+      <c r="J4" s="21" t="n"/>
+      <c r="K4" t="inlineStr">
         <is>
-          <t>Wells No.(s):         (      G-71-91        )</t>
+          <t>Wells No.(s):         (  )</t>
         </is>
       </c>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="3" t="n"/>
-      <c r="Q4" s="22" t="n"/>
     </row>
     <row r="5" ht="28.2" customHeight="1">
       <c r="A5" s="23" t="inlineStr">
@@ -1152,10 +1152,15 @@
       </c>
       <c r="J5" s="25" t="inlineStr">
         <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="K5" s="25" t="inlineStr">
+        <is>
           <t>Operations Summary</t>
         </is>
       </c>
-      <c r="Q5" s="12" t="n"/>
+      <c r="R5" s="12" t="n"/>
     </row>
     <row r="6" ht="28.2" customHeight="1">
       <c r="A6" s="26" t="n"/>
@@ -1191,8 +1196,9 @@
           <t>Operation</t>
         </is>
       </c>
-      <c r="J6" s="29" t="n"/>
-      <c r="Q6" s="12" t="n"/>
+      <c r="J6" s="26" t="n"/>
+      <c r="K6" s="29" t="n"/>
+      <c r="R6" s="12" t="n"/>
     </row>
     <row r="7" ht="28.2" customHeight="1">
       <c r="A7" s="30" t="n"/>
@@ -1236,403 +1242,255 @@
           <t>Hrs.</t>
         </is>
       </c>
-      <c r="J7" s="35" t="n"/>
-      <c r="K7" s="14" t="n"/>
+      <c r="J7" s="30" t="n"/>
+      <c r="K7" s="35" t="n"/>
       <c r="L7" s="14" t="n"/>
       <c r="M7" s="14" t="n"/>
       <c r="N7" s="14" t="n"/>
       <c r="O7" s="14" t="n"/>
       <c r="P7" s="14" t="n"/>
-      <c r="Q7" s="36" t="n"/>
-      <c r="R7" s="37" t="n"/>
+      <c r="Q7" s="14" t="n"/>
+      <c r="R7" s="36" t="n"/>
     </row>
     <row r="8" ht="26.4" customHeight="1">
-      <c r="A8" s="38" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B8" s="39" t="n">
-        <v>12</v>
-      </c>
+      <c r="A8" s="68" t="n"/>
+      <c r="B8" s="39" t="n"/>
       <c r="C8" s="39" t="n"/>
       <c r="D8" s="40" t="n"/>
       <c r="E8" s="40" t="n"/>
       <c r="F8" s="40" t="n"/>
       <c r="G8" s="40" t="n"/>
       <c r="H8" s="40" t="n"/>
-      <c r="I8" s="40">
-        <f>SUM(B8:H8)</f>
-        <v/>
-      </c>
-      <c r="J8" s="41" t="inlineStr">
-        <is>
-          <t>RIH W/DRILL STRING. DRILL OUT FILL 11FT.R/D POWER SWIVEL. POOH W/SAME IN COMPLETE</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="n"/>
+      <c r="I8" s="40" t="n"/>
+      <c r="J8" s="41" t="n"/>
+      <c r="K8" s="41" t="n"/>
       <c r="L8" s="3" t="n"/>
       <c r="M8" s="3" t="n"/>
       <c r="N8" s="3" t="n"/>
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="n"/>
-      <c r="Q8" s="22" t="n"/>
-      <c r="R8" s="37" t="n"/>
+      <c r="Q8" s="3" t="n"/>
+      <c r="R8" s="22" t="n"/>
     </row>
     <row r="9" ht="28.2" customHeight="1">
-      <c r="A9" s="38" t="n">
-        <v>46144</v>
-      </c>
-      <c r="B9" s="39" t="n">
-        <v>10</v>
-      </c>
-      <c r="C9" s="39" t="n">
-        <v>2</v>
-      </c>
+      <c r="A9" s="68" t="n"/>
+      <c r="B9" s="39" t="n"/>
+      <c r="C9" s="39" t="n"/>
       <c r="D9" s="40" t="n"/>
       <c r="E9" s="40" t="n"/>
       <c r="F9" s="40" t="n"/>
       <c r="G9" s="40" t="n"/>
       <c r="H9" s="40" t="n"/>
-      <c r="I9" s="40">
-        <f>SUM(B9:H9)</f>
-        <v/>
-      </c>
-      <c r="J9" s="42" t="inlineStr">
-        <is>
-          <t>CONT POOH W/ DRILL STRING , L/D BHA. STRIP IN C-SECTION &amp; N/UP BOPS . RIH KILL STRING. NO ENOUGH TIME TO ASSEMBLE ESP</t>
-        </is>
-      </c>
-      <c r="K9" s="43" t="n"/>
+      <c r="I9" s="40" t="n"/>
+      <c r="J9" s="42" t="n"/>
+      <c r="K9" s="42" t="n"/>
       <c r="L9" s="43" t="n"/>
       <c r="M9" s="43" t="n"/>
       <c r="N9" s="43" t="n"/>
       <c r="O9" s="43" t="n"/>
       <c r="P9" s="43" t="n"/>
-      <c r="Q9" s="44" t="n"/>
-      <c r="R9" s="37" t="n"/>
+      <c r="Q9" s="43" t="n"/>
+      <c r="R9" s="44" t="n"/>
     </row>
     <row r="10" ht="28.2" customHeight="1">
-      <c r="A10" s="38" t="n">
-        <v>46145</v>
-      </c>
-      <c r="B10" s="39" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="C10" s="39" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="A10" s="68" t="n"/>
+      <c r="B10" s="39" t="n"/>
+      <c r="C10" s="39" t="n"/>
       <c r="D10" s="40" t="n"/>
       <c r="E10" s="40" t="n"/>
       <c r="F10" s="40" t="n"/>
       <c r="G10" s="40" t="n"/>
       <c r="H10" s="40" t="n"/>
-      <c r="I10" s="40">
-        <f>SUM(B10:H10)</f>
-        <v/>
-      </c>
-      <c r="J10" s="42" t="inlineStr">
-        <is>
-          <t>POOH W/KILL STRING . WAIT ON ESP TEC . ASSMBLE ESP . SLIP 15 FT DRILL LINE . RIH W/ESP INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="K10" s="43" t="n"/>
+      <c r="I10" s="40" t="n"/>
+      <c r="J10" s="42" t="n"/>
+      <c r="K10" s="42" t="n"/>
       <c r="L10" s="43" t="n"/>
       <c r="M10" s="43" t="n"/>
       <c r="N10" s="43" t="n"/>
       <c r="O10" s="43" t="n"/>
       <c r="P10" s="43" t="n"/>
-      <c r="Q10" s="44" t="n"/>
+      <c r="Q10" s="43" t="n"/>
+      <c r="R10" s="44" t="n"/>
     </row>
     <row r="11" ht="28.2" customHeight="1">
-      <c r="A11" s="38" t="n">
-        <v>46146</v>
-      </c>
-      <c r="B11" s="39" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="C11" s="39" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="A11" s="68" t="n"/>
+      <c r="B11" s="39" t="n"/>
+      <c r="C11" s="39" t="n"/>
       <c r="D11" s="40" t="n"/>
       <c r="E11" s="40" t="n"/>
       <c r="F11" s="40" t="n"/>
       <c r="G11" s="40" t="n"/>
       <c r="H11" s="40" t="n"/>
-      <c r="I11" s="40">
-        <f>SUM(B11:H11)</f>
-        <v/>
-      </c>
-      <c r="J11" s="42" t="inlineStr">
-        <is>
-          <t>CONT RIH W/ESP. NO ENOUGH TIME TO SPLICE</t>
-        </is>
-      </c>
-      <c r="K11" s="43" t="n"/>
+      <c r="I11" s="40" t="n"/>
+      <c r="J11" s="42" t="n"/>
+      <c r="K11" s="42" t="n"/>
       <c r="L11" s="43" t="n"/>
       <c r="M11" s="43" t="n"/>
       <c r="N11" s="43" t="n"/>
       <c r="O11" s="43" t="n"/>
       <c r="P11" s="43" t="n"/>
-      <c r="Q11" s="44" t="n"/>
-      <c r="R11" s="37" t="n"/>
+      <c r="Q11" s="43" t="n"/>
+      <c r="R11" s="44" t="n"/>
     </row>
     <row r="12" ht="28.2" customHeight="1">
-      <c r="A12" s="38" t="n">
-        <v>46147</v>
-      </c>
-      <c r="B12" s="39" t="n">
-        <v>3</v>
-      </c>
-      <c r="C12" s="39" t="n">
-        <v>9</v>
-      </c>
+      <c r="A12" s="68" t="n"/>
+      <c r="B12" s="39" t="n"/>
+      <c r="C12" s="39" t="n"/>
       <c r="D12" s="40" t="n"/>
       <c r="E12" s="40" t="n"/>
       <c r="F12" s="40" t="n"/>
       <c r="G12" s="40" t="n"/>
       <c r="H12" s="40" t="n"/>
-      <c r="I12" s="40">
-        <f>SUM(B12:H12)</f>
-        <v/>
-      </c>
-      <c r="J12" s="42" t="inlineStr">
-        <is>
-          <t>SPLICE LOWER PIG TAIL . N/D BOP , N/UP W.H. HOOK UP ELECT START UP ESP TO STATION OVER NIGHT</t>
-        </is>
-      </c>
-      <c r="K12" s="43" t="n"/>
+      <c r="I12" s="40" t="n"/>
+      <c r="J12" s="42" t="n"/>
+      <c r="K12" s="42" t="n"/>
       <c r="L12" s="43" t="n"/>
       <c r="M12" s="43" t="n"/>
       <c r="N12" s="43" t="n"/>
       <c r="O12" s="43" t="n"/>
       <c r="P12" s="43" t="n"/>
-      <c r="Q12" s="44" t="n"/>
-      <c r="R12" s="37" t="n"/>
+      <c r="Q12" s="43" t="n"/>
+      <c r="R12" s="44" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="38" t="n">
-        <v>46148</v>
-      </c>
+      <c r="A13" s="68" t="n"/>
       <c r="B13" s="39" t="n"/>
-      <c r="C13" s="39" t="n">
-        <v>12</v>
-      </c>
+      <c r="C13" s="39" t="n"/>
       <c r="D13" s="40" t="n"/>
       <c r="E13" s="40" t="n"/>
       <c r="F13" s="40" t="n"/>
       <c r="G13" s="40" t="n"/>
       <c r="H13" s="40" t="n"/>
-      <c r="I13" s="40">
-        <f>SUM(B13:H13)</f>
-        <v/>
-      </c>
-      <c r="J13" s="42" t="inlineStr">
-        <is>
-          <t>CONT TEST WELL FLOWING TO STATION OVER NIGHT</t>
-        </is>
-      </c>
-      <c r="K13" s="43" t="n"/>
+      <c r="I13" s="40" t="n"/>
+      <c r="J13" s="42" t="n"/>
+      <c r="K13" s="42" t="n"/>
       <c r="L13" s="43" t="n"/>
       <c r="M13" s="43" t="n"/>
       <c r="N13" s="43" t="n"/>
       <c r="O13" s="43" t="n"/>
       <c r="P13" s="43" t="n"/>
-      <c r="Q13" s="44" t="n"/>
-      <c r="R13" s="37" t="n"/>
+      <c r="Q13" s="43" t="n"/>
+      <c r="R13" s="44" t="n"/>
     </row>
     <row r="14" ht="24.6" customHeight="1">
-      <c r="A14" s="38" t="n">
-        <v>46149</v>
-      </c>
+      <c r="A14" s="68" t="n"/>
       <c r="B14" s="39" t="n"/>
-      <c r="C14" s="39" t="n">
-        <v>12</v>
-      </c>
+      <c r="C14" s="39" t="n"/>
       <c r="D14" s="40" t="n"/>
       <c r="E14" s="40" t="n"/>
       <c r="F14" s="40" t="n"/>
       <c r="G14" s="40" t="n"/>
       <c r="H14" s="40" t="n"/>
-      <c r="I14" s="40">
-        <f>SUM(B14:H14)</f>
-        <v/>
-      </c>
-      <c r="J14" s="42" t="inlineStr">
-        <is>
-          <t>CONT TEST WELL FLOWING TO STATION W/ NESR SEP OVER NIGHT</t>
-        </is>
-      </c>
-      <c r="K14" s="43" t="n"/>
+      <c r="I14" s="40" t="n"/>
+      <c r="J14" s="42" t="n"/>
+      <c r="K14" s="42" t="n"/>
       <c r="L14" s="43" t="n"/>
       <c r="M14" s="43" t="n"/>
       <c r="N14" s="43" t="n"/>
       <c r="O14" s="43" t="n"/>
       <c r="P14" s="43" t="n"/>
-      <c r="Q14" s="44" t="n"/>
-      <c r="R14" s="37" t="n"/>
+      <c r="Q14" s="43" t="n"/>
+      <c r="R14" s="44" t="n"/>
     </row>
     <row r="15" ht="26.4" customHeight="1">
-      <c r="A15" s="38" t="n">
-        <v>46150</v>
-      </c>
+      <c r="A15" s="68" t="n"/>
       <c r="B15" s="39" t="n"/>
-      <c r="C15" s="39" t="n">
-        <v>12</v>
-      </c>
+      <c r="C15" s="39" t="n"/>
       <c r="D15" s="40" t="n"/>
       <c r="E15" s="40" t="n"/>
       <c r="F15" s="40" t="n"/>
       <c r="G15" s="40" t="n"/>
       <c r="H15" s="40" t="n"/>
-      <c r="I15" s="40">
-        <f>SUM(B15:H15)</f>
-        <v/>
-      </c>
-      <c r="J15" s="42" t="inlineStr">
-        <is>
-          <t>CONT TEST WELL FLOWING TO STATION OVER NIGHT</t>
-        </is>
-      </c>
-      <c r="K15" s="43" t="n"/>
+      <c r="I15" s="40" t="n"/>
+      <c r="J15" s="42" t="n"/>
+      <c r="K15" s="42" t="n"/>
       <c r="L15" s="43" t="n"/>
       <c r="M15" s="43" t="n"/>
       <c r="N15" s="43" t="n"/>
       <c r="O15" s="43" t="n"/>
       <c r="P15" s="43" t="n"/>
-      <c r="Q15" s="44" t="n"/>
-      <c r="R15" s="37" t="n"/>
+      <c r="Q15" s="43" t="n"/>
+      <c r="R15" s="44" t="n"/>
     </row>
     <row r="16" ht="25.2" customHeight="1">
-      <c r="A16" s="38" t="n">
-        <v>46151</v>
-      </c>
+      <c r="A16" s="68" t="n"/>
       <c r="B16" s="39" t="n"/>
-      <c r="C16" s="39" t="n">
-        <v>12</v>
-      </c>
+      <c r="C16" s="39" t="n"/>
       <c r="D16" s="39" t="n"/>
       <c r="E16" s="39" t="n"/>
       <c r="F16" s="39" t="n"/>
       <c r="G16" s="39" t="n"/>
       <c r="H16" s="39" t="n"/>
-      <c r="I16" s="40">
-        <f>SUM(B16:H16)</f>
-        <v/>
-      </c>
-      <c r="J16" s="42" t="inlineStr">
-        <is>
-          <t>CONT TEST WELL FLOWING TO STATION OVER NIGHT</t>
-        </is>
-      </c>
-      <c r="K16" s="43" t="n"/>
+      <c r="I16" s="40" t="n"/>
+      <c r="J16" s="42" t="n"/>
+      <c r="K16" s="42" t="n"/>
       <c r="L16" s="43" t="n"/>
       <c r="M16" s="43" t="n"/>
       <c r="N16" s="43" t="n"/>
       <c r="O16" s="43" t="n"/>
       <c r="P16" s="43" t="n"/>
-      <c r="Q16" s="44" t="n"/>
+      <c r="Q16" s="43" t="n"/>
+      <c r="R16" s="44" t="n"/>
     </row>
     <row r="17" ht="24.6" customHeight="1">
-      <c r="A17" s="38" t="n">
-        <v>46152</v>
-      </c>
+      <c r="A17" s="68" t="n"/>
       <c r="B17" s="39" t="n"/>
-      <c r="C17" s="39" t="n">
-        <v>4.5</v>
-      </c>
+      <c r="C17" s="39" t="n"/>
       <c r="D17" s="45" t="n"/>
       <c r="E17" s="39" t="n"/>
       <c r="F17" s="39" t="n"/>
       <c r="G17" s="39" t="n"/>
-      <c r="H17" s="39" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="I17" s="40">
-        <f>SUM(B17:H17)</f>
-        <v/>
-      </c>
-      <c r="J17" s="46" t="inlineStr">
-        <is>
-          <t>CONT TEST WELL FLOWING TO STATION . R/D RIG 100% &amp; MOVE OUT LOC 40%</t>
-        </is>
-      </c>
-      <c r="K17" s="47" t="n"/>
+      <c r="H17" s="39" t="n"/>
+      <c r="I17" s="40" t="n"/>
+      <c r="J17" s="46" t="n"/>
+      <c r="K17" s="46" t="n"/>
       <c r="L17" s="47" t="n"/>
       <c r="M17" s="47" t="n"/>
       <c r="N17" s="47" t="n"/>
       <c r="O17" s="47" t="n"/>
       <c r="P17" s="47" t="n"/>
-      <c r="Q17" s="48" t="n"/>
+      <c r="Q17" s="47" t="n"/>
+      <c r="R17" s="48" t="n"/>
     </row>
     <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="38" t="n">
-        <v>46153</v>
-      </c>
+      <c r="A18" s="68" t="n"/>
       <c r="B18" s="39" t="n"/>
       <c r="C18" s="39" t="n"/>
       <c r="D18" s="39" t="n"/>
       <c r="E18" s="39" t="n"/>
-      <c r="F18" s="39" t="n">
-        <v>1</v>
-      </c>
+      <c r="F18" s="39" t="n"/>
       <c r="G18" s="39" t="n"/>
-      <c r="H18" s="39" t="n">
-        <v>6</v>
-      </c>
-      <c r="I18" s="40">
-        <f>SUM(B18:H18)</f>
-        <v/>
-      </c>
-      <c r="J18" s="42" t="inlineStr">
-        <is>
-          <t>CONT MOVE OUT LOCATION 100% &amp; CLEAN , LEVEL LOCATION 100%</t>
-        </is>
-      </c>
-      <c r="K18" s="43" t="n"/>
+      <c r="H18" s="39" t="n"/>
+      <c r="I18" s="40" t="n"/>
+      <c r="J18" s="42" t="n"/>
+      <c r="K18" s="42" t="n"/>
       <c r="L18" s="43" t="n"/>
       <c r="M18" s="43" t="n"/>
       <c r="N18" s="43" t="n"/>
       <c r="O18" s="43" t="n"/>
       <c r="P18" s="43" t="n"/>
-      <c r="Q18" s="44" t="n"/>
-      <c r="R18" s="37" t="n"/>
+      <c r="Q18" s="43" t="n"/>
+      <c r="R18" s="44" t="n"/>
     </row>
     <row r="19" ht="28.2" customHeight="1">
-      <c r="A19" s="38" t="n"/>
-      <c r="B19" s="40">
-        <f>SUM(B8:B18)</f>
-        <v/>
-      </c>
-      <c r="C19" s="40">
-        <f>SUM(C8:C18)</f>
-        <v/>
-      </c>
+      <c r="A19" s="68" t="n"/>
+      <c r="B19" s="40" t="n"/>
+      <c r="C19" s="40" t="n"/>
       <c r="D19" s="40" t="n"/>
-      <c r="E19" s="40">
-        <f>SUM(E8:E18)</f>
-        <v/>
-      </c>
-      <c r="F19" s="40">
-        <f>SUM(F8:F18)</f>
-        <v/>
-      </c>
+      <c r="E19" s="40" t="n"/>
+      <c r="F19" s="40" t="n"/>
       <c r="G19" s="40" t="n"/>
-      <c r="H19" s="40">
-        <f>SUM(H8:H18)</f>
-        <v/>
-      </c>
-      <c r="I19" s="40">
-        <f>SUM(I8:I18)</f>
-        <v/>
-      </c>
+      <c r="H19" s="40" t="n"/>
+      <c r="I19" s="40" t="n"/>
       <c r="J19" s="49" t="n"/>
-      <c r="K19" s="10" t="n"/>
+      <c r="K19" s="49" t="n"/>
       <c r="L19" s="10" t="n"/>
       <c r="M19" s="10" t="n"/>
       <c r="N19" s="10" t="n"/>
       <c r="O19" s="10" t="n"/>
       <c r="P19" s="10" t="n"/>
-      <c r="Q19" s="50" t="n"/>
-      <c r="R19" s="37" t="n"/>
+      <c r="Q19" s="10" t="n"/>
+      <c r="R19" s="50" t="n"/>
     </row>
     <row r="20" ht="28.2" customHeight="1">
       <c r="A20" s="51" t="inlineStr">
@@ -1648,11 +1506,11 @@
       <c r="G20" s="10" t="n"/>
       <c r="H20" s="10" t="n"/>
       <c r="I20" s="10" t="n"/>
-      <c r="Q20" s="12" t="n"/>
+      <c r="R20" s="12" t="n"/>
     </row>
     <row r="21" ht="28.2" customHeight="1">
       <c r="A21" s="29" t="n"/>
-      <c r="Q21" s="12" t="n"/>
+      <c r="R21" s="12" t="n"/>
     </row>
     <row r="22" ht="28.2" customHeight="1">
       <c r="A22" s="35" t="n"/>
@@ -1664,60 +1522,70 @@
       <c r="G22" s="14" t="n"/>
       <c r="H22" s="14" t="n"/>
       <c r="I22" s="14" t="n"/>
-      <c r="J22" s="14" t="n"/>
       <c r="K22" s="14" t="n"/>
       <c r="L22" s="14" t="n"/>
       <c r="M22" s="14" t="n"/>
       <c r="N22" s="14" t="n"/>
       <c r="O22" s="14" t="n"/>
       <c r="P22" s="14" t="n"/>
-      <c r="Q22" s="36" t="n"/>
+      <c r="Q22" s="14" t="n"/>
+      <c r="R22" s="36" t="n"/>
     </row>
     <row r="23" ht="28.2" customHeight="1">
       <c r="J23" s="45" t="n"/>
+      <c r="K23" s="45" t="n"/>
     </row>
     <row r="24" ht="28.2" customHeight="1">
       <c r="J24" s="45" t="n"/>
+      <c r="K24" s="45" t="n"/>
     </row>
     <row r="25" ht="28.2" customHeight="1">
       <c r="C25" s="52" t="n"/>
       <c r="J25" s="45" t="n"/>
+      <c r="K25" s="45" t="n"/>
     </row>
     <row r="26" ht="28.2" customHeight="1">
       <c r="J26" s="53" t="n"/>
+      <c r="K26" s="53" t="n"/>
     </row>
     <row r="27" ht="28.2" customHeight="1">
       <c r="J27" s="45" t="n"/>
+      <c r="K27" s="45" t="n"/>
     </row>
     <row r="28" ht="28.2" customHeight="1">
       <c r="J28" s="54" t="n"/>
-      <c r="Q28" s="55" t="n"/>
+      <c r="K28" s="54" t="n"/>
+      <c r="R28" s="55" t="n"/>
     </row>
     <row r="29" ht="28.2" customHeight="1">
       <c r="J29" s="53" t="n"/>
+      <c r="K29" s="53" t="n"/>
     </row>
     <row r="30" ht="28.2" customHeight="1">
       <c r="J30" s="56" t="n"/>
-      <c r="K30" s="57" t="n"/>
+      <c r="K30" s="56" t="n"/>
       <c r="L30" s="57" t="n"/>
       <c r="M30" s="57" t="n"/>
       <c r="N30" s="57" t="n"/>
       <c r="O30" s="57" t="n"/>
       <c r="P30" s="57" t="n"/>
-      <c r="Q30" s="58" t="n"/>
+      <c r="Q30" s="57" t="n"/>
+      <c r="R30" s="58" t="n"/>
     </row>
     <row r="31" ht="28.2" customHeight="1">
       <c r="J31" s="59" t="n"/>
+      <c r="K31" s="59" t="n"/>
     </row>
     <row r="32" ht="28.2" customHeight="1">
       <c r="J32" s="60" t="n"/>
-      <c r="K32" s="57" t="n"/>
+      <c r="K32" s="60" t="n"/>
       <c r="L32" s="57" t="n"/>
       <c r="M32" s="57" t="n"/>
       <c r="N32" s="57" t="n"/>
       <c r="O32" s="57" t="n"/>
       <c r="P32" s="57" t="n"/>
-      <c r="Q32" s="58" t="n"/>
+      <c r="Q32" s="57" t="n"/>
+      <c r="R32" s="58" t="n"/>
     </row>
     <row r="33" ht="28.2" customHeight="1">
       <c r="C33" s="61" t="n"/>
@@ -1726,21 +1594,24 @@
       <c r="H33" s="61" t="n"/>
       <c r="I33" s="62" t="n"/>
       <c r="J33" s="63" t="n"/>
-      <c r="K33" s="64" t="n"/>
+      <c r="K33" s="63" t="n"/>
       <c r="L33" s="64" t="n"/>
       <c r="M33" s="64" t="n"/>
       <c r="N33" s="64" t="n"/>
       <c r="O33" s="64" t="n"/>
       <c r="P33" s="64" t="n"/>
-      <c r="Q33" s="65" t="n"/>
+      <c r="Q33" s="64" t="n"/>
+      <c r="R33" s="65" t="n"/>
     </row>
     <row r="34" ht="28.2" customHeight="1">
       <c r="D34" s="66" t="n"/>
       <c r="I34" s="66" t="n"/>
       <c r="J34" s="59" t="n"/>
+      <c r="K34" s="59" t="n"/>
     </row>
     <row r="35" ht="28.2" customHeight="1">
       <c r="J35" s="45" t="n"/>
+      <c r="K35" s="45" t="n"/>
     </row>
     <row r="36" ht="28.2" customHeight="1">
       <c r="C36" s="67" t="n"/>
@@ -1751,6 +1622,7 @@
       <c r="H36" s="67" t="n"/>
       <c r="I36" s="67" t="n"/>
       <c r="J36" s="67" t="n"/>
+      <c r="K36" s="67" t="n"/>
     </row>
     <row r="37" ht="28.2" customHeight="1">
       <c r="C37" s="67" t="n"/>
@@ -1761,6 +1633,7 @@
       <c r="H37" s="67" t="n"/>
       <c r="I37" s="67" t="n"/>
       <c r="J37" s="67" t="n"/>
+      <c r="K37" s="67" t="n"/>
     </row>
     <row r="38" ht="28.2" customHeight="1">
       <c r="C38" s="67" t="n"/>
@@ -1771,6 +1644,7 @@
       <c r="H38" s="67" t="n"/>
       <c r="I38" s="67" t="n"/>
       <c r="J38" s="45" t="n"/>
+      <c r="K38" s="45" t="n"/>
     </row>
     <row r="39" ht="28.2" customHeight="1">
       <c r="C39" s="67" t="n"/>
@@ -1781,6 +1655,7 @@
       <c r="H39" s="67" t="n"/>
       <c r="I39" s="67" t="n"/>
       <c r="J39" s="67" t="n"/>
+      <c r="K39" s="67" t="n"/>
     </row>
     <row r="40" ht="28.2" customHeight="1">
       <c r="J40" s="45" t="n"/>
@@ -7465,38 +7340,39 @@
       <c r="J1933" s="45" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="31">
-    <mergeCell ref="J8:Q8"/>
+  <mergeCells count="32">
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="J14:Q14"/>
-    <mergeCell ref="J29:Q29"/>
+    <mergeCell ref="K16:R16"/>
+    <mergeCell ref="K30:R30"/>
+    <mergeCell ref="K15:R15"/>
+    <mergeCell ref="K33:R33"/>
     <mergeCell ref="A5:A7"/>
-    <mergeCell ref="J5:Q7"/>
-    <mergeCell ref="J10:Q10"/>
-    <mergeCell ref="J28:Q28"/>
-    <mergeCell ref="J13:Q13"/>
+    <mergeCell ref="K2:R3"/>
+    <mergeCell ref="K9:R9"/>
     <mergeCell ref="B5:H5"/>
-    <mergeCell ref="J9:Q9"/>
-    <mergeCell ref="J30:Q30"/>
-    <mergeCell ref="J15:Q15"/>
-    <mergeCell ref="J2:Q3"/>
+    <mergeCell ref="K26:R26"/>
+    <mergeCell ref="K29:R29"/>
+    <mergeCell ref="K11:R11"/>
+    <mergeCell ref="K5:R7"/>
+    <mergeCell ref="K32:R32"/>
     <mergeCell ref="B1:F1"/>
+    <mergeCell ref="J5:J7"/>
+    <mergeCell ref="K19:R22"/>
     <mergeCell ref="A20:I22"/>
     <mergeCell ref="E6:F6"/>
-    <mergeCell ref="J4:Q4"/>
-    <mergeCell ref="J26:Q26"/>
-    <mergeCell ref="J11:Q11"/>
-    <mergeCell ref="J16:Q16"/>
-    <mergeCell ref="J32:Q32"/>
+    <mergeCell ref="K12:R12"/>
+    <mergeCell ref="K8:R8"/>
+    <mergeCell ref="K14:R14"/>
+    <mergeCell ref="K17:R17"/>
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="C33:E33"/>
-    <mergeCell ref="J12:Q12"/>
     <mergeCell ref="B2:I3"/>
     <mergeCell ref="C4:E4"/>
-    <mergeCell ref="J33:Q33"/>
-    <mergeCell ref="J19:Q22"/>
-    <mergeCell ref="J18:Q18"/>
-    <mergeCell ref="J17:Q17"/>
+    <mergeCell ref="K10:R10"/>
+    <mergeCell ref="K28:R28"/>
+    <mergeCell ref="K4:R4"/>
+    <mergeCell ref="K13:R13"/>
+    <mergeCell ref="K18:R18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>